<commit_message>
Set stall stock (50/40/30/20) and updated Idly/Rose Milk prices in projection
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RGZwPX49EKhhzekY9w6486
</commit_message>
<xml_diff>
--- a/stall/Stall_Sales_Projection.xlsx
+++ b/stall/Stall_Sales_Projection.xlsx
@@ -87,7 +87,7 @@
     <t xml:space="preserve">1 plate</t>
   </si>
   <si>
-    <t xml:space="preserve">Prices: from you.</t>
+    <t xml:space="preserve">Prices: from you (Idly $8 and Rose Milk $4, as updated in the tracker).</t>
   </si>
   <si>
     <t xml:space="preserve">Paneer Puff</t>
@@ -102,7 +102,7 @@
     <t xml:space="preserve">Podi Idly</t>
   </si>
   <si>
-    <t xml:space="preserve">Stock: placeholder. Enter how many you're making for the weekend.</t>
+    <t xml:space="preserve">Stock: from you (50 / 40 / 30 / 20 for the weekend).</t>
   </si>
   <si>
     <t xml:space="preserve">Rose Milk</t>
@@ -471,16 +471,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -492,99 +496,99 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -885,280 +889,280 @@
   <dimension ref="A1:I21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="70"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="F5" s="8" t="n">
+      <c r="D5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="F5" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="F6" s="8" t="n">
+      <c r="D6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>40</v>
+      </c>
+      <c r="F6" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>45</v>
-      </c>
-      <c r="F7" s="8" t="n">
+      <c r="C7" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="D7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>70</v>
-      </c>
-      <c r="F8" s="8" t="n">
+      <c r="C8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="F8" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
       <c r="E9" s="9"/>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9"/>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
       <c r="E10" s="9"/>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="B16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="13" t="n">
         <f aca="false">SUM(B13:B16)</f>
         <v>160</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
         <v>33</v>
       </c>
       <c r="B20" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="8" t="n">
+      <c r="B21" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="3" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1182,487 +1186,487 @@
   <dimension ref="A1:H26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="str">
         <f aca="false">IF(Inputs!A5="","",Inputs!A5)</f>
         <v>Medhu Vadai</v>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B5" s="15" t="n">
         <f aca="false">Inputs!C5</f>
         <v>6</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="16" t="n">
         <f aca="false">Inputs!F5*Inputs!$B$20</f>
         <v>20</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="17" t="n">
         <f aca="false">C5*$B5</f>
         <v>120</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="16" t="n">
         <f aca="false">Inputs!G5*Inputs!$B$20</f>
         <v>40</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="17" t="n">
         <f aca="false">E5*$B5</f>
         <v>240</v>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="16" t="n">
         <f aca="false">Inputs!H5*Inputs!$B$20</f>
         <v>70</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="17" t="n">
         <f aca="false">G5*$B5</f>
         <v>420</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="str">
         <f aca="false">IF(Inputs!A6="","",Inputs!A6)</f>
         <v>Paneer Puff</v>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="15" t="n">
         <f aca="false">Inputs!C6</f>
         <v>4</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <f aca="false">Inputs!F6*Inputs!$B$20</f>
         <v>20</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="17" t="n">
         <f aca="false">C6*$B6</f>
         <v>80</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="16" t="n">
         <f aca="false">Inputs!G6*Inputs!$B$20</f>
         <v>40</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="17" t="n">
         <f aca="false">E6*$B6</f>
         <v>160</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="16" t="n">
         <f aca="false">Inputs!H6*Inputs!$B$20</f>
         <v>70</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <f aca="false">G6*$B6</f>
         <v>280</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="str">
         <f aca="false">IF(Inputs!A7="","",Inputs!A7)</f>
         <v>Podi Idly</v>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="15" t="n">
         <f aca="false">Inputs!C7</f>
-        <v>6</v>
-      </c>
-      <c r="C7" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="16" t="n">
         <f aca="false">Inputs!F7*Inputs!$B$20</f>
         <v>16</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="17" t="n">
         <f aca="false">C7*$B7</f>
-        <v>96</v>
-      </c>
-      <c r="E7" s="15" t="n">
+        <v>128</v>
+      </c>
+      <c r="E7" s="16" t="n">
         <f aca="false">Inputs!G7*Inputs!$B$20</f>
         <v>30</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="17" t="n">
         <f aca="false">E7*$B7</f>
-        <v>180</v>
-      </c>
-      <c r="G7" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="G7" s="16" t="n">
         <f aca="false">Inputs!H7*Inputs!$B$20</f>
         <v>50</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="17" t="n">
         <f aca="false">G7*$B7</f>
-        <v>300</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="str">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="str">
         <f aca="false">IF(Inputs!A8="","",Inputs!A8)</f>
         <v>Rose Milk</v>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="15" t="n">
         <f aca="false">Inputs!C8</f>
-        <v>5</v>
-      </c>
-      <c r="C8" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="16" t="n">
         <f aca="false">Inputs!F8*Inputs!$B$20</f>
         <v>24</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">C8*$B8</f>
-        <v>120</v>
-      </c>
-      <c r="E8" s="15" t="n">
+        <v>96</v>
+      </c>
+      <c r="E8" s="16" t="n">
         <f aca="false">Inputs!G8*Inputs!$B$20</f>
         <v>50</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="17" t="n">
         <f aca="false">E8*$B8</f>
-        <v>250</v>
-      </c>
-      <c r="G8" s="15" t="n">
+        <v>200</v>
+      </c>
+      <c r="G8" s="16" t="n">
         <f aca="false">Inputs!H8*Inputs!$B$20</f>
         <v>80</v>
       </c>
-      <c r="H8" s="16" t="n">
+      <c r="H8" s="17" t="n">
         <f aca="false">G8*$B8</f>
-        <v>400</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="str">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="str">
         <f aca="false">IF(Inputs!A9="","",Inputs!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="15" t="n">
         <f aca="false">Inputs!C9</f>
         <v>0</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <f aca="false">Inputs!F9*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <f aca="false">C9*$B9</f>
         <v>0</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="16" t="n">
         <f aca="false">Inputs!G9*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="17" t="n">
         <f aca="false">E9*$B9</f>
         <v>0</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="16" t="n">
         <f aca="false">Inputs!H9*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="H9" s="16" t="n">
+      <c r="H9" s="17" t="n">
         <f aca="false">G9*$B9</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="str">
         <f aca="false">IF(Inputs!A10="","",Inputs!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="14" t="n">
+      <c r="B10" s="15" t="n">
         <f aca="false">Inputs!C10</f>
         <v>0</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <f aca="false">Inputs!F10*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="17" t="n">
         <f aca="false">C10*$B10</f>
         <v>0</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="16" t="n">
         <f aca="false">Inputs!G10*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="17" t="n">
         <f aca="false">E10*$B10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="15" t="n">
+      <c r="G10" s="16" t="n">
         <f aca="false">Inputs!H10*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="H10" s="16" t="n">
+      <c r="H10" s="17" t="n">
         <f aca="false">G10*$B10</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="19" t="n">
+      <c r="B11" s="19"/>
+      <c r="C11" s="20" t="n">
         <f aca="false">SUM(C5:C10)</f>
         <v>80</v>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="21" t="n">
         <f aca="false">SUM(D5:D10)</f>
-        <v>416</v>
-      </c>
-      <c r="E11" s="19" t="n">
+        <v>424</v>
+      </c>
+      <c r="E11" s="20" t="n">
         <f aca="false">SUM(E5:E10)</f>
         <v>160</v>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="21" t="n">
         <f aca="false">SUM(F5:F10)</f>
-        <v>830</v>
-      </c>
-      <c r="G11" s="19" t="n">
+        <v>840</v>
+      </c>
+      <c r="G11" s="20" t="n">
         <f aca="false">SUM(G5:G10)</f>
         <v>270</v>
       </c>
-      <c r="H11" s="20" t="n">
+      <c r="H11" s="21" t="n">
         <f aca="false">SUM(H5:H10)</f>
-        <v>1400</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="16" t="n">
+      <c r="B14" s="17" t="n">
         <f aca="false">D11</f>
-        <v>416</v>
-      </c>
-      <c r="C14" s="16" t="n">
+        <v>424</v>
+      </c>
+      <c r="C14" s="17" t="n">
         <f aca="false">F11</f>
-        <v>830</v>
-      </c>
-      <c r="D14" s="16" t="n">
+        <v>840</v>
+      </c>
+      <c r="D14" s="17" t="n">
         <f aca="false">H11</f>
-        <v>1400</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
+        <v>1420</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="16" t="n">
+      <c r="B15" s="17" t="n">
         <f aca="false">SUMPRODUCT(C5:C10,Inputs!$D$5:$D$10)</f>
         <v>0</v>
       </c>
-      <c r="C15" s="16" t="n">
+      <c r="C15" s="17" t="n">
         <f aca="false">SUMPRODUCT(E5:E10,Inputs!$D$5:$D$10)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="16" t="n">
+      <c r="D15" s="17" t="n">
         <f aca="false">SUMPRODUCT(G5:G10,Inputs!$D$5:$D$10)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="22" t="n">
         <f aca="false">Inputs!$B$17</f>
         <v>160</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="22" t="n">
         <f aca="false">Inputs!$B$17</f>
         <v>160</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="22" t="n">
         <f aca="false">Inputs!$B$17</f>
         <v>160</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="20" t="n">
+      <c r="B17" s="21" t="n">
         <f aca="false">B14-B15-B16</f>
-        <v>256</v>
-      </c>
-      <c r="C17" s="20" t="n">
+        <v>264</v>
+      </c>
+      <c r="C17" s="21" t="n">
         <f aca="false">C14-C15-C16</f>
-        <v>670</v>
-      </c>
-      <c r="D17" s="20" t="n">
+        <v>680</v>
+      </c>
+      <c r="D17" s="21" t="n">
         <f aca="false">D14-D15-D16</f>
-        <v>1240</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="22" t="n">
+      <c r="B18" s="23" t="n">
         <f aca="false">IF(B14=0,0,B17/B14)</f>
-        <v>0.615384615384615</v>
-      </c>
-      <c r="C18" s="22" t="n">
+        <v>0.622641509433962</v>
+      </c>
+      <c r="C18" s="23" t="n">
         <f aca="false">IF(C14=0,0,C17/C14)</f>
-        <v>0.807228915662651</v>
-      </c>
-      <c r="D18" s="22" t="n">
+        <v>0.80952380952381</v>
+      </c>
+      <c r="D18" s="23" t="n">
         <f aca="false">IF(D14=0,0,D17/D14)</f>
-        <v>0.885714285714286</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+        <v>0.887323943661972</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="23" t="n">
+      <c r="B19" s="24" t="n">
         <f aca="false">C11</f>
         <v>80</v>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="24" t="n">
         <f aca="false">E11</f>
         <v>160</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="24" t="n">
         <f aca="false">G11</f>
         <v>270</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="24" t="n">
+      <c r="B20" s="25" t="n">
         <f aca="false">IF(Inputs!$B$20*Inputs!$B$21=0,0,B19/(Inputs!$B$20*Inputs!$B$21))</f>
         <v>6.66666666666667</v>
       </c>
-      <c r="C20" s="24" t="n">
+      <c r="C20" s="25" t="n">
         <f aca="false">IF(Inputs!$B$20*Inputs!$B$21=0,0,C19/(Inputs!$B$20*Inputs!$B$21))</f>
         <v>13.3333333333333</v>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D20" s="25" t="n">
         <f aca="false">IF(Inputs!$B$20*Inputs!$B$21=0,0,D19/(Inputs!$B$20*Inputs!$B$21))</f>
         <v>22.5</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="25" t="n">
+      <c r="B21" s="26" t="n">
         <f aca="false">IF(B19=0,0,B14/B19)</f>
-        <v>5.2</v>
-      </c>
-      <c r="C21" s="25" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="C21" s="26" t="n">
         <f aca="false">IF(C19=0,0,C14/C19)</f>
-        <v>5.1875</v>
-      </c>
-      <c r="D21" s="25" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="D21" s="26" t="n">
         <f aca="false">IF(D19=0,0,D14/D19)</f>
-        <v>5.18518518518519</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
+        <v>5.25925925925926</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="25" t="n">
+      <c r="B22" s="26" t="n">
         <f aca="false">IF(B19=0,0,(B14-B15)/B19)</f>
-        <v>5.2</v>
-      </c>
-      <c r="C22" s="25" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="C22" s="26" t="n">
         <f aca="false">IF(C19=0,0,(C14-C15)/C19)</f>
-        <v>5.1875</v>
-      </c>
-      <c r="D22" s="25" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="D22" s="26" t="n">
         <f aca="false">IF(D19=0,0,(D14-D15)/D19)</f>
-        <v>5.18518518518519</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
+        <v>5.25925925925926</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="23" t="n">
+      <c r="B23" s="24" t="n">
         <f aca="false">IF(B22&lt;=0,0,ROUNDUP(Inputs!$B$17/B22,0))</f>
         <v>31</v>
       </c>
-      <c r="C23" s="23" t="n">
+      <c r="C23" s="24" t="n">
         <f aca="false">IF(C22&lt;=0,0,ROUNDUP(Inputs!$B$17/C22,0))</f>
         <v>31</v>
       </c>
-      <c r="D23" s="23" t="n">
+      <c r="D23" s="24" t="n">
         <f aca="false">IF(D22&lt;=0,0,ROUNDUP(Inputs!$B$17/D22,0))</f>
         <v>31</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="16" t="n">
+      <c r="B24" s="17" t="n">
         <f aca="false">B23*B21</f>
-        <v>161.2</v>
-      </c>
-      <c r="C24" s="16" t="n">
+        <v>164.3</v>
+      </c>
+      <c r="C24" s="17" t="n">
         <f aca="false">C23*C21</f>
-        <v>160.8125</v>
-      </c>
-      <c r="D24" s="16" t="n">
+        <v>162.75</v>
+      </c>
+      <c r="D24" s="17" t="n">
         <f aca="false">D23*D21</f>
-        <v>160.740740740741</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+        <v>163.037037037037</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1693,322 +1697,322 @@
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="26" t="n">
+      <c r="B4" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="26" t="n">
+      <c r="C4" s="27" t="n">
         <v>4.5</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="D4" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="26" t="n">
+      <c r="E4" s="27" t="n">
         <v>5.5</v>
       </c>
-      <c r="F4" s="26" t="n">
+      <c r="F4" s="27" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <f aca="false">$A5*$B$18*(B$4-$B$16)-$B$17</f>
         <v>-80</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <f aca="false">$A5*$B$18*(C$4-$B$16)-$B$17</f>
         <v>-70</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="17" t="n">
         <f aca="false">$A5*$B$18*(D$4-$B$16)-$B$17</f>
         <v>-60</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="17" t="n">
         <f aca="false">$A5*$B$18*(E$4-$B$16)-$B$17</f>
         <v>-50</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="17" t="n">
         <f aca="false">$A5*$B$18*(F$4-$B$16)-$B$17</f>
         <v>-40</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="27" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="28" t="n">
         <v>20</v>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="17" t="n">
         <f aca="false">$A6*$B$18*(B$4-$B$16)-$B$17</f>
         <v>0</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="17" t="n">
         <f aca="false">$A6*$B$18*(C$4-$B$16)-$B$17</f>
         <v>20</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="17" t="n">
         <f aca="false">$A6*$B$18*(D$4-$B$16)-$B$17</f>
         <v>40</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="17" t="n">
         <f aca="false">$A6*$B$18*(E$4-$B$16)-$B$17</f>
         <v>60</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="17" t="n">
         <f aca="false">$A6*$B$18*(F$4-$B$16)-$B$17</f>
         <v>80</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="n">
         <v>30</v>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="17" t="n">
         <f aca="false">$A7*$B$18*(B$4-$B$16)-$B$17</f>
         <v>80</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="17" t="n">
         <f aca="false">$A7*$B$18*(C$4-$B$16)-$B$17</f>
         <v>110</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="17" t="n">
         <f aca="false">$A7*$B$18*(D$4-$B$16)-$B$17</f>
         <v>140</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="17" t="n">
         <f aca="false">$A7*$B$18*(E$4-$B$16)-$B$17</f>
         <v>170</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="17" t="n">
         <f aca="false">$A7*$B$18*(F$4-$B$16)-$B$17</f>
         <v>200</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="27" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="28" t="n">
         <v>40</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="17" t="n">
         <f aca="false">$A8*$B$18*(B$4-$B$16)-$B$17</f>
         <v>160</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="17" t="n">
         <f aca="false">$A8*$B$18*(C$4-$B$16)-$B$17</f>
         <v>200</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">$A8*$B$18*(D$4-$B$16)-$B$17</f>
         <v>240</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="17" t="n">
         <f aca="false">$A8*$B$18*(E$4-$B$16)-$B$17</f>
         <v>280</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="17" t="n">
         <f aca="false">$A8*$B$18*(F$4-$B$16)-$B$17</f>
         <v>320</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="27" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="28" t="n">
         <v>50</v>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="17" t="n">
         <f aca="false">$A9*$B$18*(B$4-$B$16)-$B$17</f>
         <v>240</v>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="17" t="n">
         <f aca="false">$A9*$B$18*(C$4-$B$16)-$B$17</f>
         <v>290</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <f aca="false">$A9*$B$18*(D$4-$B$16)-$B$17</f>
         <v>340</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="17" t="n">
         <f aca="false">$A9*$B$18*(E$4-$B$16)-$B$17</f>
         <v>390</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="17" t="n">
         <f aca="false">$A9*$B$18*(F$4-$B$16)-$B$17</f>
         <v>440</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="27" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="28" t="n">
         <v>60</v>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="17" t="n">
         <f aca="false">$A10*$B$18*(B$4-$B$16)-$B$17</f>
         <v>320</v>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="17" t="n">
         <f aca="false">$A10*$B$18*(C$4-$B$16)-$B$17</f>
         <v>380</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="17" t="n">
         <f aca="false">$A10*$B$18*(D$4-$B$16)-$B$17</f>
         <v>440</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="17" t="n">
         <f aca="false">$A10*$B$18*(E$4-$B$16)-$B$17</f>
         <v>500</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="17" t="n">
         <f aca="false">$A10*$B$18*(F$4-$B$16)-$B$17</f>
         <v>560</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="28" t="n">
         <v>70</v>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B11" s="17" t="n">
         <f aca="false">$A11*$B$18*(B$4-$B$16)-$B$17</f>
         <v>400</v>
       </c>
-      <c r="C11" s="16" t="n">
+      <c r="C11" s="17" t="n">
         <f aca="false">$A11*$B$18*(C$4-$B$16)-$B$17</f>
         <v>470</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="17" t="n">
         <f aca="false">$A11*$B$18*(D$4-$B$16)-$B$17</f>
         <v>540</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="17" t="n">
         <f aca="false">$A11*$B$18*(E$4-$B$16)-$B$17</f>
         <v>610</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="17" t="n">
         <f aca="false">$A11*$B$18*(F$4-$B$16)-$B$17</f>
         <v>680</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="27" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="28" t="n">
         <v>80</v>
       </c>
-      <c r="B12" s="16" t="n">
+      <c r="B12" s="17" t="n">
         <f aca="false">$A12*$B$18*(B$4-$B$16)-$B$17</f>
         <v>480</v>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="17" t="n">
         <f aca="false">$A12*$B$18*(C$4-$B$16)-$B$17</f>
         <v>560</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="17" t="n">
         <f aca="false">$A12*$B$18*(D$4-$B$16)-$B$17</f>
         <v>640</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="17" t="n">
         <f aca="false">$A12*$B$18*(E$4-$B$16)-$B$17</f>
         <v>720</v>
       </c>
-      <c r="F12" s="16" t="n">
+      <c r="F12" s="17" t="n">
         <f aca="false">$A12*$B$18*(F$4-$B$16)-$B$17</f>
         <v>800</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="27" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="28" t="n">
         <v>90</v>
       </c>
-      <c r="B13" s="16" t="n">
+      <c r="B13" s="17" t="n">
         <f aca="false">$A13*$B$18*(B$4-$B$16)-$B$17</f>
         <v>560</v>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="17" t="n">
         <f aca="false">$A13*$B$18*(C$4-$B$16)-$B$17</f>
         <v>650</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="17" t="n">
         <f aca="false">$A13*$B$18*(D$4-$B$16)-$B$17</f>
         <v>740</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E13" s="17" t="n">
         <f aca="false">$A13*$B$18*(E$4-$B$16)-$B$17</f>
         <v>830</v>
       </c>
-      <c r="F13" s="16" t="n">
+      <c r="F13" s="17" t="n">
         <f aca="false">$A13*$B$18*(F$4-$B$16)-$B$17</f>
         <v>920</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="27" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="B14" s="16" t="n">
+      <c r="B14" s="17" t="n">
         <f aca="false">$A14*$B$18*(B$4-$B$16)-$B$17</f>
         <v>640</v>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="17" t="n">
         <f aca="false">$A14*$B$18*(C$4-$B$16)-$B$17</f>
         <v>740</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="17" t="n">
         <f aca="false">$A14*$B$18*(D$4-$B$16)-$B$17</f>
         <v>840</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="17" t="n">
         <f aca="false">$A14*$B$18*(E$4-$B$16)-$B$17</f>
         <v>940</v>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F14" s="17" t="n">
         <f aca="false">$A14*$B$18*(F$4-$B$16)-$B$17</f>
         <v>1040</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="14" t="n">
+      <c r="B16" s="15" t="n">
         <f aca="false">IF(Projection!C19=0,0,Projection!C15/Projection!C19)</f>
         <v>0</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="22" t="n">
         <f aca="false">Inputs!B17</f>
         <v>160</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="15" t="n">
+      <c r="B18" s="16" t="n">
         <f aca="false">Inputs!B20</f>
         <v>2</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>66</v>
       </c>
     </row>
@@ -2039,255 +2043,255 @@
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="32"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="str">
         <f aca="false">IF(Inputs!A5="","",Inputs!A5)</f>
         <v>Medhu Vadai</v>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="16" t="n">
         <f aca="false">Inputs!E5</f>
-        <v>60</v>
-      </c>
-      <c r="C5" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="C5" s="16" t="n">
         <f aca="false">Projection!E5</f>
         <v>40</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="16" t="n">
         <f aca="false">Projection!G5</f>
         <v>70</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="24" t="n">
         <f aca="false">IF(OR(A5="",Inputs!E5=""),0,B5-C5)</f>
-        <v>20</v>
-      </c>
-      <c r="F5" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" s="17" t="n">
         <f aca="false">B5*Inputs!C5</f>
-        <v>360</v>
-      </c>
-      <c r="G5" s="10" t="str">
+        <v>300</v>
+      </c>
+      <c r="G5" s="11" t="str">
         <f aca="false">IF(A5="","",IF(Inputs!E5="","Enter stock on Inputs",IF(B5&gt;=D5,"Enough even for a busy weekend",IF(B5&gt;=C5,"Enough for expected","Short by "&amp;(C5-B5)&amp;" for expected"))))</f>
         <v>Enough for expected</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="str">
         <f aca="false">IF(Inputs!A6="","",Inputs!A6)</f>
         <v>Paneer Puff</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="16" t="n">
         <f aca="false">Inputs!E6</f>
-        <v>60</v>
-      </c>
-      <c r="C6" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="C6" s="16" t="n">
         <f aca="false">Projection!E6</f>
         <v>40</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="16" t="n">
         <f aca="false">Projection!G6</f>
         <v>70</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="24" t="n">
         <f aca="false">IF(OR(A6="",Inputs!E6=""),0,B6-C6)</f>
-        <v>20</v>
-      </c>
-      <c r="F6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="17" t="n">
         <f aca="false">B6*Inputs!C6</f>
-        <v>240</v>
-      </c>
-      <c r="G6" s="10" t="str">
+        <v>160</v>
+      </c>
+      <c r="G6" s="11" t="str">
         <f aca="false">IF(A6="","",IF(Inputs!E6="","Enter stock on Inputs",IF(B6&gt;=D6,"Enough even for a busy weekend",IF(B6&gt;=C6,"Enough for expected","Short by "&amp;(C6-B6)&amp;" for expected"))))</f>
         <v>Enough for expected</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="str">
         <f aca="false">IF(Inputs!A7="","",Inputs!A7)</f>
         <v>Podi Idly</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="16" t="n">
         <f aca="false">Inputs!E7</f>
-        <v>45</v>
-      </c>
-      <c r="C7" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="C7" s="16" t="n">
         <f aca="false">Projection!E7</f>
         <v>30</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="16" t="n">
         <f aca="false">Projection!G7</f>
         <v>50</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="24" t="n">
         <f aca="false">IF(OR(A7="",Inputs!E7=""),0,B7-C7)</f>
-        <v>15</v>
-      </c>
-      <c r="F7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="17" t="n">
         <f aca="false">B7*Inputs!C7</f>
-        <v>270</v>
-      </c>
-      <c r="G7" s="10" t="str">
+        <v>240</v>
+      </c>
+      <c r="G7" s="11" t="str">
         <f aca="false">IF(A7="","",IF(Inputs!E7="","Enter stock on Inputs",IF(B7&gt;=D7,"Enough even for a busy weekend",IF(B7&gt;=C7,"Enough for expected","Short by "&amp;(C7-B7)&amp;" for expected"))))</f>
         <v>Enough for expected</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="str">
         <f aca="false">IF(Inputs!A8="","",Inputs!A8)</f>
         <v>Rose Milk</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="16" t="n">
         <f aca="false">Inputs!E8</f>
-        <v>70</v>
-      </c>
-      <c r="C8" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" s="16" t="n">
         <f aca="false">Projection!E8</f>
         <v>50</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="16" t="n">
         <f aca="false">Projection!G8</f>
         <v>80</v>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E8" s="24" t="n">
         <f aca="false">IF(OR(A8="",Inputs!E8=""),0,B8-C8)</f>
-        <v>20</v>
-      </c>
-      <c r="F8" s="16" t="n">
+        <v>-30</v>
+      </c>
+      <c r="F8" s="17" t="n">
         <f aca="false">B8*Inputs!C8</f>
-        <v>350</v>
-      </c>
-      <c r="G8" s="10" t="str">
+        <v>80</v>
+      </c>
+      <c r="G8" s="11" t="str">
         <f aca="false">IF(A8="","",IF(Inputs!E8="","Enter stock on Inputs",IF(B8&gt;=D8,"Enough even for a busy weekend",IF(B8&gt;=C8,"Enough for expected","Short by "&amp;(C8-B8)&amp;" for expected"))))</f>
-        <v>Enough for expected</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="str">
+        <v>Short by 30 for expected</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="str">
         <f aca="false">IF(Inputs!A9="","",Inputs!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="16" t="n">
         <f aca="false">Inputs!E9</f>
         <v>0</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <f aca="false">Projection!E9</f>
         <v>0</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="16" t="n">
         <f aca="false">Projection!G9</f>
         <v>0</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="24" t="n">
         <f aca="false">IF(OR(A9="",Inputs!E9=""),0,B9-C9)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="17" t="n">
         <f aca="false">B9*Inputs!C9</f>
         <v>0</v>
       </c>
-      <c r="G9" s="10" t="str">
+      <c r="G9" s="11" t="str">
         <f aca="false">IF(A9="","",IF(Inputs!E9="","Enter stock on Inputs",IF(B9&gt;=D9,"Enough even for a busy weekend",IF(B9&gt;=C9,"Enough for expected","Short by "&amp;(C9-B9)&amp;" for expected"))))</f>
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="str">
         <f aca="false">IF(Inputs!A10="","",Inputs!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="16" t="n">
         <f aca="false">Inputs!E10</f>
         <v>0</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <f aca="false">Projection!E10</f>
         <v>0</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="16" t="n">
         <f aca="false">Projection!G10</f>
         <v>0</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="24" t="n">
         <f aca="false">IF(OR(A10="",Inputs!E10=""),0,B10-C10)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="17" t="n">
         <f aca="false">B10*Inputs!C10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="10" t="str">
+      <c r="G10" s="11" t="str">
         <f aca="false">IF(A10="","",IF(Inputs!E10="","Enter stock on Inputs",IF(B10&gt;=D10,"Enough even for a busy weekend",IF(B10&gt;=C10,"Enough for expected","Short by "&amp;(C10-B10)&amp;" for expected"))))</f>
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="20" t="n">
         <f aca="false">SUM(B5:B10)</f>
-        <v>235</v>
-      </c>
-      <c r="C11" s="19" t="n">
+        <v>140</v>
+      </c>
+      <c r="C11" s="20" t="n">
         <f aca="false">SUM(C5:C10)</f>
         <v>160</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="20" t="n">
         <f aca="false">SUM(D5:D10)</f>
         <v>270</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="20" t="n">
         <f aca="false">SUM(E5:E10)</f>
-        <v>75</v>
-      </c>
-      <c r="F11" s="20" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F11" s="21" t="n">
         <f aca="false">SUM(F5:F10)</f>
-        <v>1220</v>
-      </c>
-      <c r="G11" s="18"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+        <v>780</v>
+      </c>
+      <c r="G11" s="19"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2315,285 +2319,285 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="str">
         <f aca="false">IF(Inputs!A5="","",Inputs!A5)</f>
         <v>Medhu Vadai</v>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="16" t="n">
         <f aca="false">Projection!E5</f>
         <v>40</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="24" t="n">
         <f aca="false">IF(C5="",0,C5-B5)</f>
         <v>-22</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="22" t="n">
         <f aca="false">Projection!F5</f>
         <v>240</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="17" t="n">
         <f aca="false">N(C5)*Inputs!C5</f>
         <v>108</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="str">
         <f aca="false">IF(Inputs!A6="","",Inputs!A6)</f>
         <v>Paneer Puff</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="16" t="n">
         <f aca="false">Projection!E6</f>
         <v>40</v>
       </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="23" t="n">
+      <c r="C6" s="10"/>
+      <c r="D6" s="24" t="n">
         <f aca="false">IF(C6="",0,C6-B6)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="22" t="n">
         <f aca="false">Projection!F6</f>
         <v>160</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="17" t="n">
         <f aca="false">N(C6)*Inputs!C6</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="str">
         <f aca="false">IF(Inputs!A7="","",Inputs!A7)</f>
         <v>Podi Idly</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="16" t="n">
         <f aca="false">Projection!E7</f>
         <v>30</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="23" t="n">
+      <c r="C7" s="10"/>
+      <c r="D7" s="24" t="n">
         <f aca="false">IF(C7="",0,C7-B7)</f>
         <v>0</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="22" t="n">
         <f aca="false">Projection!F7</f>
-        <v>180</v>
-      </c>
-      <c r="F7" s="16" t="n">
+        <v>240</v>
+      </c>
+      <c r="F7" s="17" t="n">
         <f aca="false">N(C7)*Inputs!C7</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="str">
         <f aca="false">IF(Inputs!A8="","",Inputs!A8)</f>
         <v>Rose Milk</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="16" t="n">
         <f aca="false">Projection!E8</f>
         <v>50</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="23" t="n">
+      <c r="C8" s="10"/>
+      <c r="D8" s="24" t="n">
         <f aca="false">IF(C8="",0,C8-B8)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="22" t="n">
         <f aca="false">Projection!F8</f>
-        <v>250</v>
-      </c>
-      <c r="F8" s="16" t="n">
+        <v>200</v>
+      </c>
+      <c r="F8" s="17" t="n">
         <f aca="false">N(C8)*Inputs!C8</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="str">
         <f aca="false">IF(Inputs!A9="","",Inputs!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="16" t="n">
         <f aca="false">Projection!E9</f>
         <v>0</v>
       </c>
       <c r="C9" s="9"/>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="24" t="n">
         <f aca="false">IF(C9="",0,C9-B9)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="22" t="n">
         <f aca="false">Projection!F9</f>
         <v>0</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="17" t="n">
         <f aca="false">N(C9)*Inputs!C9</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="str">
         <f aca="false">IF(Inputs!A10="","",Inputs!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="16" t="n">
         <f aca="false">Projection!E10</f>
         <v>0</v>
       </c>
       <c r="C10" s="9"/>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="24" t="n">
         <f aca="false">IF(C10="",0,C10-B10)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="22" t="n">
         <f aca="false">Projection!F10</f>
         <v>0</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="17" t="n">
         <f aca="false">N(C10)*Inputs!C10</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="20" t="n">
         <f aca="false">SUM(B5:B10)</f>
         <v>160</v>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C11" s="20" t="n">
         <f aca="false">SUM(C5:C10)</f>
         <v>18</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="20" t="n">
         <f aca="false">SUM(D5:D10)</f>
         <v>-22</v>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="21" t="n">
         <f aca="false">SUM(E5:E10)</f>
-        <v>830</v>
-      </c>
-      <c r="F11" s="20" t="n">
+        <v>840</v>
+      </c>
+      <c r="F11" s="21" t="n">
         <f aca="false">SUM(F5:F10)</f>
         <v>108</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="16" t="n">
+      <c r="B14" s="17" t="n">
         <f aca="false">E11</f>
-        <v>830</v>
-      </c>
-      <c r="C14" s="16" t="n">
+        <v>840</v>
+      </c>
+      <c r="C14" s="17" t="n">
         <f aca="false">F11</f>
         <v>108</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="21" t="n">
+      <c r="B15" s="22" t="n">
         <f aca="false">Projection!C15</f>
         <v>0</v>
       </c>
-      <c r="C15" s="16" t="n">
+      <c r="C15" s="17" t="n">
         <f aca="false">SUMPRODUCT(C5:C10,Inputs!$D$5:$D$10)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="22" t="n">
         <f aca="false">Inputs!B17</f>
         <v>160</v>
       </c>
-      <c r="C16" s="28" t="n">
+      <c r="C16" s="29" t="n">
         <f aca="false">Inputs!B17</f>
         <v>160</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="20" t="n">
+      <c r="B17" s="21" t="n">
         <f aca="false">B14-B15-B16</f>
-        <v>670</v>
-      </c>
-      <c r="C17" s="20" t="n">
+        <v>680</v>
+      </c>
+      <c r="C17" s="21" t="n">
         <f aca="false">C14-C15-C16</f>
         <v>-52</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="C18" s="16" t="n">
+      <c r="C18" s="17" t="n">
         <f aca="false">C17-B17</f>
-        <v>-722</v>
+        <v>-732</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Show price column and compute actual sales as price x units sold
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RGZwPX49EKhhzekY9w6486
</commit_message>
<xml_diff>
--- a/stall/Stall_Sales_Projection.xlsx
+++ b/stall/Stall_Sales_Projection.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="85">
   <si>
     <t xml:space="preserve">Snack Stall: Projection Inputs</t>
   </si>
@@ -273,19 +273,17 @@
     <t xml:space="preserve">Actuals vs Projection</t>
   </si>
   <si>
-    <t xml:space="preserve">After the weekend, enter units sold from the tracker's Summary export (the Sold column). Yellow cells are yours to fill.</t>
+    <t xml:space="preserve">After the weekend, enter units sold from the tracker's Summary export (the Sold column). Actual sales = price x units sold. Yellow cells are yours to fill.</t>
   </si>
   <si>
     <t xml:space="preserve">Actual units sold</t>
   </si>
   <si>
-    <t xml:space="preserve">Difference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Actual sales ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example value. Replace with your real number.</t>
+    <t xml:space="preserve">Difference (units)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actual sales ($)
+= price x units</t>
   </si>
   <si>
     <t xml:space="preserve">Profit</t>
@@ -301,6 +299,9 @@
   </si>
   <si>
     <t xml:space="preserve">Actual vs expected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leave Actual units blank until the weekend is done. Until then, Actual shows a loss of your spend.</t>
   </si>
 </sst>
 </file>
@@ -471,20 +472,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -496,99 +493,99 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -889,280 +886,280 @@
   <dimension ref="A1:I21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="70"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="9" t="n">
+      <c r="D5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G5" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H5" s="9" t="n">
         <v>35</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="9" t="n">
+      <c r="D6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="H6" s="10" t="n">
+      <c r="H6" s="9" t="n">
         <v>35</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="D7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="9" t="n">
+      <c r="D7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="9" t="n">
+      <c r="D8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="G8" s="10" t="n">
+      <c r="G8" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="H8" s="10" t="n">
+      <c r="H8" s="9" t="n">
         <v>40</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I8" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="10" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="3" t="s">
+      <c r="B16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="13" t="n">
+      <c r="B17" s="12" t="n">
         <f aca="false">SUM(B13:B16)</f>
         <v>160</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B20" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="2" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1186,487 +1183,487 @@
   <dimension ref="A1:H26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="str">
         <f aca="false">IF(Inputs!A5="","",Inputs!A5)</f>
         <v>Medhu Vadai</v>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="14" t="n">
         <f aca="false">Inputs!C5</f>
         <v>6</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="15" t="n">
         <f aca="false">Inputs!F5*Inputs!$B$20</f>
         <v>20</v>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="16" t="n">
         <f aca="false">C5*$B5</f>
         <v>120</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="15" t="n">
         <f aca="false">Inputs!G5*Inputs!$B$20</f>
         <v>40</v>
       </c>
-      <c r="F5" s="17" t="n">
+      <c r="F5" s="16" t="n">
         <f aca="false">E5*$B5</f>
         <v>240</v>
       </c>
-      <c r="G5" s="16" t="n">
+      <c r="G5" s="15" t="n">
         <f aca="false">Inputs!H5*Inputs!$B$20</f>
         <v>70</v>
       </c>
-      <c r="H5" s="17" t="n">
+      <c r="H5" s="16" t="n">
         <f aca="false">G5*$B5</f>
         <v>420</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="str">
         <f aca="false">IF(Inputs!A6="","",Inputs!A6)</f>
         <v>Paneer Puff</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="14" t="n">
         <f aca="false">Inputs!C6</f>
         <v>4</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="15" t="n">
         <f aca="false">Inputs!F6*Inputs!$B$20</f>
         <v>20</v>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="16" t="n">
         <f aca="false">C6*$B6</f>
         <v>80</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="15" t="n">
         <f aca="false">Inputs!G6*Inputs!$B$20</f>
         <v>40</v>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="16" t="n">
         <f aca="false">E6*$B6</f>
         <v>160</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="15" t="n">
         <f aca="false">Inputs!H6*Inputs!$B$20</f>
         <v>70</v>
       </c>
-      <c r="H6" s="17" t="n">
+      <c r="H6" s="16" t="n">
         <f aca="false">G6*$B6</f>
         <v>280</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="str">
         <f aca="false">IF(Inputs!A7="","",Inputs!A7)</f>
         <v>Podi Idly</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="14" t="n">
         <f aca="false">Inputs!C7</f>
         <v>8</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="15" t="n">
         <f aca="false">Inputs!F7*Inputs!$B$20</f>
         <v>16</v>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="16" t="n">
         <f aca="false">C7*$B7</f>
         <v>128</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="15" t="n">
         <f aca="false">Inputs!G7*Inputs!$B$20</f>
         <v>30</v>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="F7" s="16" t="n">
         <f aca="false">E7*$B7</f>
         <v>240</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="15" t="n">
         <f aca="false">Inputs!H7*Inputs!$B$20</f>
         <v>50</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="H7" s="16" t="n">
         <f aca="false">G7*$B7</f>
         <v>400</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="str">
         <f aca="false">IF(Inputs!A8="","",Inputs!A8)</f>
         <v>Rose Milk</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="14" t="n">
         <f aca="false">Inputs!C8</f>
         <v>4</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="15" t="n">
         <f aca="false">Inputs!F8*Inputs!$B$20</f>
         <v>24</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="16" t="n">
         <f aca="false">C8*$B8</f>
         <v>96</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="15" t="n">
         <f aca="false">Inputs!G8*Inputs!$B$20</f>
         <v>50</v>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="F8" s="16" t="n">
         <f aca="false">E8*$B8</f>
         <v>200</v>
       </c>
-      <c r="G8" s="16" t="n">
+      <c r="G8" s="15" t="n">
         <f aca="false">Inputs!H8*Inputs!$B$20</f>
         <v>80</v>
       </c>
-      <c r="H8" s="17" t="n">
+      <c r="H8" s="16" t="n">
         <f aca="false">G8*$B8</f>
         <v>320</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="str">
         <f aca="false">IF(Inputs!A9="","",Inputs!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="14" t="n">
         <f aca="false">Inputs!C9</f>
         <v>0</v>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="15" t="n">
         <f aca="false">Inputs!F9*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="16" t="n">
         <f aca="false">C9*$B9</f>
         <v>0</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="15" t="n">
         <f aca="false">Inputs!G9*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="F9" s="16" t="n">
         <f aca="false">E9*$B9</f>
         <v>0</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="G9" s="15" t="n">
         <f aca="false">Inputs!H9*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="H9" s="17" t="n">
+      <c r="H9" s="16" t="n">
         <f aca="false">G9*$B9</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="str">
         <f aca="false">IF(Inputs!A10="","",Inputs!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="14" t="n">
         <f aca="false">Inputs!C10</f>
         <v>0</v>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="15" t="n">
         <f aca="false">Inputs!F10*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="16" t="n">
         <f aca="false">C10*$B10</f>
         <v>0</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="15" t="n">
         <f aca="false">Inputs!G10*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="F10" s="17" t="n">
+      <c r="F10" s="16" t="n">
         <f aca="false">E10*$B10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G10" s="15" t="n">
         <f aca="false">Inputs!H10*Inputs!$B$20</f>
         <v>0</v>
       </c>
-      <c r="H10" s="17" t="n">
+      <c r="H10" s="16" t="n">
         <f aca="false">G10*$B10</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="20" t="n">
+      <c r="B11" s="18"/>
+      <c r="C11" s="19" t="n">
         <f aca="false">SUM(C5:C10)</f>
         <v>80</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="20" t="n">
         <f aca="false">SUM(D5:D10)</f>
         <v>424</v>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="19" t="n">
         <f aca="false">SUM(E5:E10)</f>
         <v>160</v>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" s="20" t="n">
         <f aca="false">SUM(F5:F10)</f>
         <v>840</v>
       </c>
-      <c r="G11" s="20" t="n">
+      <c r="G11" s="19" t="n">
         <f aca="false">SUM(G5:G10)</f>
         <v>270</v>
       </c>
-      <c r="H11" s="21" t="n">
+      <c r="H11" s="20" t="n">
         <f aca="false">SUM(H5:H10)</f>
         <v>1420</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="16" t="n">
         <f aca="false">D11</f>
         <v>424</v>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="16" t="n">
         <f aca="false">F11</f>
         <v>840</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="16" t="n">
         <f aca="false">H11</f>
         <v>1420</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B15" s="16" t="n">
         <f aca="false">SUMPRODUCT(C5:C10,Inputs!$D$5:$D$10)</f>
         <v>0</v>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="16" t="n">
         <f aca="false">SUMPRODUCT(E5:E10,Inputs!$D$5:$D$10)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="D15" s="16" t="n">
         <f aca="false">SUMPRODUCT(G5:G10,Inputs!$D$5:$D$10)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="21" t="n">
         <f aca="false">Inputs!$B$17</f>
         <v>160</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="21" t="n">
         <f aca="false">Inputs!$B$17</f>
         <v>160</v>
       </c>
-      <c r="D16" s="22" t="n">
+      <c r="D16" s="21" t="n">
         <f aca="false">Inputs!$B$17</f>
         <v>160</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="20" t="n">
         <f aca="false">B14-B15-B16</f>
         <v>264</v>
       </c>
-      <c r="C17" s="21" t="n">
+      <c r="C17" s="20" t="n">
         <f aca="false">C14-C15-C16</f>
         <v>680</v>
       </c>
-      <c r="D17" s="21" t="n">
+      <c r="D17" s="20" t="n">
         <f aca="false">D14-D15-D16</f>
         <v>1260</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="23" t="n">
+      <c r="B18" s="22" t="n">
         <f aca="false">IF(B14=0,0,B17/B14)</f>
         <v>0.622641509433962</v>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="22" t="n">
         <f aca="false">IF(C14=0,0,C17/C14)</f>
         <v>0.80952380952381</v>
       </c>
-      <c r="D18" s="23" t="n">
+      <c r="D18" s="22" t="n">
         <f aca="false">IF(D14=0,0,D17/D14)</f>
         <v>0.887323943661972</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="24" t="n">
+      <c r="B19" s="23" t="n">
         <f aca="false">C11</f>
         <v>80</v>
       </c>
-      <c r="C19" s="24" t="n">
+      <c r="C19" s="23" t="n">
         <f aca="false">E11</f>
         <v>160</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="23" t="n">
         <f aca="false">G11</f>
         <v>270</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="25" t="n">
+      <c r="B20" s="24" t="n">
         <f aca="false">IF(Inputs!$B$20*Inputs!$B$21=0,0,B19/(Inputs!$B$20*Inputs!$B$21))</f>
         <v>6.66666666666667</v>
       </c>
-      <c r="C20" s="25" t="n">
+      <c r="C20" s="24" t="n">
         <f aca="false">IF(Inputs!$B$20*Inputs!$B$21=0,0,C19/(Inputs!$B$20*Inputs!$B$21))</f>
         <v>13.3333333333333</v>
       </c>
-      <c r="D20" s="25" t="n">
+      <c r="D20" s="24" t="n">
         <f aca="false">IF(Inputs!$B$20*Inputs!$B$21=0,0,D19/(Inputs!$B$20*Inputs!$B$21))</f>
         <v>22.5</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="25" t="n">
         <f aca="false">IF(B19=0,0,B14/B19)</f>
         <v>5.3</v>
       </c>
-      <c r="C21" s="26" t="n">
+      <c r="C21" s="25" t="n">
         <f aca="false">IF(C19=0,0,C14/C19)</f>
         <v>5.25</v>
       </c>
-      <c r="D21" s="26" t="n">
+      <c r="D21" s="25" t="n">
         <f aca="false">IF(D19=0,0,D14/D19)</f>
         <v>5.25925925925926</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="26" t="n">
+      <c r="B22" s="25" t="n">
         <f aca="false">IF(B19=0,0,(B14-B15)/B19)</f>
         <v>5.3</v>
       </c>
-      <c r="C22" s="26" t="n">
+      <c r="C22" s="25" t="n">
         <f aca="false">IF(C19=0,0,(C14-C15)/C19)</f>
         <v>5.25</v>
       </c>
-      <c r="D22" s="26" t="n">
+      <c r="D22" s="25" t="n">
         <f aca="false">IF(D19=0,0,(D14-D15)/D19)</f>
         <v>5.25925925925926</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="24" t="n">
+      <c r="B23" s="23" t="n">
         <f aca="false">IF(B22&lt;=0,0,ROUNDUP(Inputs!$B$17/B22,0))</f>
         <v>31</v>
       </c>
-      <c r="C23" s="24" t="n">
+      <c r="C23" s="23" t="n">
         <f aca="false">IF(C22&lt;=0,0,ROUNDUP(Inputs!$B$17/C22,0))</f>
         <v>31</v>
       </c>
-      <c r="D23" s="24" t="n">
+      <c r="D23" s="23" t="n">
         <f aca="false">IF(D22&lt;=0,0,ROUNDUP(Inputs!$B$17/D22,0))</f>
         <v>31</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="17" t="n">
+      <c r="B24" s="16" t="n">
         <f aca="false">B23*B21</f>
         <v>164.3</v>
       </c>
-      <c r="C24" s="17" t="n">
+      <c r="C24" s="16" t="n">
         <f aca="false">C23*C21</f>
         <v>162.75</v>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="D24" s="16" t="n">
         <f aca="false">D23*D21</f>
         <v>163.037037037037</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1697,322 +1694,322 @@
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="27" t="n">
+      <c r="B4" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="27" t="n">
+      <c r="C4" s="26" t="n">
         <v>4.5</v>
       </c>
-      <c r="D4" s="27" t="n">
+      <c r="D4" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="27" t="n">
+      <c r="E4" s="26" t="n">
         <v>5.5</v>
       </c>
-      <c r="F4" s="27" t="n">
+      <c r="F4" s="26" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="16" t="n">
         <f aca="false">$A5*$B$18*(B$4-$B$16)-$B$17</f>
         <v>-80</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="16" t="n">
         <f aca="false">$A5*$B$18*(C$4-$B$16)-$B$17</f>
         <v>-70</v>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="16" t="n">
         <f aca="false">$A5*$B$18*(D$4-$B$16)-$B$17</f>
         <v>-60</v>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="16" t="n">
         <f aca="false">$A5*$B$18*(E$4-$B$16)-$B$17</f>
         <v>-50</v>
       </c>
-      <c r="F5" s="17" t="n">
+      <c r="F5" s="16" t="n">
         <f aca="false">$A5*$B$18*(F$4-$B$16)-$B$17</f>
         <v>-40</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="16" t="n">
         <f aca="false">$A6*$B$18*(B$4-$B$16)-$B$17</f>
         <v>0</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="16" t="n">
         <f aca="false">$A6*$B$18*(C$4-$B$16)-$B$17</f>
         <v>20</v>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="16" t="n">
         <f aca="false">$A6*$B$18*(D$4-$B$16)-$B$17</f>
         <v>40</v>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="16" t="n">
         <f aca="false">$A6*$B$18*(E$4-$B$16)-$B$17</f>
         <v>60</v>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="16" t="n">
         <f aca="false">$A6*$B$18*(F$4-$B$16)-$B$17</f>
         <v>80</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="16" t="n">
         <f aca="false">$A7*$B$18*(B$4-$B$16)-$B$17</f>
         <v>80</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="16" t="n">
         <f aca="false">$A7*$B$18*(C$4-$B$16)-$B$17</f>
         <v>110</v>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="16" t="n">
         <f aca="false">$A7*$B$18*(D$4-$B$16)-$B$17</f>
         <v>140</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="16" t="n">
         <f aca="false">$A7*$B$18*(E$4-$B$16)-$B$17</f>
         <v>170</v>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="F7" s="16" t="n">
         <f aca="false">$A7*$B$18*(F$4-$B$16)-$B$17</f>
         <v>200</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="27" t="n">
         <v>40</v>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="16" t="n">
         <f aca="false">$A8*$B$18*(B$4-$B$16)-$B$17</f>
         <v>160</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="16" t="n">
         <f aca="false">$A8*$B$18*(C$4-$B$16)-$B$17</f>
         <v>200</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="16" t="n">
         <f aca="false">$A8*$B$18*(D$4-$B$16)-$B$17</f>
         <v>240</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="16" t="n">
         <f aca="false">$A8*$B$18*(E$4-$B$16)-$B$17</f>
         <v>280</v>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="F8" s="16" t="n">
         <f aca="false">$A8*$B$18*(F$4-$B$16)-$B$17</f>
         <v>320</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="27" t="n">
         <v>50</v>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="16" t="n">
         <f aca="false">$A9*$B$18*(B$4-$B$16)-$B$17</f>
         <v>240</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="16" t="n">
         <f aca="false">$A9*$B$18*(C$4-$B$16)-$B$17</f>
         <v>290</v>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="16" t="n">
         <f aca="false">$A9*$B$18*(D$4-$B$16)-$B$17</f>
         <v>340</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="16" t="n">
         <f aca="false">$A9*$B$18*(E$4-$B$16)-$B$17</f>
         <v>390</v>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="F9" s="16" t="n">
         <f aca="false">$A9*$B$18*(F$4-$B$16)-$B$17</f>
         <v>440</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="27" t="n">
         <v>60</v>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="16" t="n">
         <f aca="false">$A10*$B$18*(B$4-$B$16)-$B$17</f>
         <v>320</v>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="16" t="n">
         <f aca="false">$A10*$B$18*(C$4-$B$16)-$B$17</f>
         <v>380</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="16" t="n">
         <f aca="false">$A10*$B$18*(D$4-$B$16)-$B$17</f>
         <v>440</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="16" t="n">
         <f aca="false">$A10*$B$18*(E$4-$B$16)-$B$17</f>
         <v>500</v>
       </c>
-      <c r="F10" s="17" t="n">
+      <c r="F10" s="16" t="n">
         <f aca="false">$A10*$B$18*(F$4-$B$16)-$B$17</f>
         <v>560</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="27" t="n">
         <v>70</v>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="16" t="n">
         <f aca="false">$A11*$B$18*(B$4-$B$16)-$B$17</f>
         <v>400</v>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="16" t="n">
         <f aca="false">$A11*$B$18*(C$4-$B$16)-$B$17</f>
         <v>470</v>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="D11" s="16" t="n">
         <f aca="false">$A11*$B$18*(D$4-$B$16)-$B$17</f>
         <v>540</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="16" t="n">
         <f aca="false">$A11*$B$18*(E$4-$B$16)-$B$17</f>
         <v>610</v>
       </c>
-      <c r="F11" s="17" t="n">
+      <c r="F11" s="16" t="n">
         <f aca="false">$A11*$B$18*(F$4-$B$16)-$B$17</f>
         <v>680</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="27" t="n">
         <v>80</v>
       </c>
-      <c r="B12" s="17" t="n">
+      <c r="B12" s="16" t="n">
         <f aca="false">$A12*$B$18*(B$4-$B$16)-$B$17</f>
         <v>480</v>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="16" t="n">
         <f aca="false">$A12*$B$18*(C$4-$B$16)-$B$17</f>
         <v>560</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="16" t="n">
         <f aca="false">$A12*$B$18*(D$4-$B$16)-$B$17</f>
         <v>640</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="16" t="n">
         <f aca="false">$A12*$B$18*(E$4-$B$16)-$B$17</f>
         <v>720</v>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="F12" s="16" t="n">
         <f aca="false">$A12*$B$18*(F$4-$B$16)-$B$17</f>
         <v>800</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="27" t="n">
         <v>90</v>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="16" t="n">
         <f aca="false">$A13*$B$18*(B$4-$B$16)-$B$17</f>
         <v>560</v>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C13" s="16" t="n">
         <f aca="false">$A13*$B$18*(C$4-$B$16)-$B$17</f>
         <v>650</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="16" t="n">
         <f aca="false">$A13*$B$18*(D$4-$B$16)-$B$17</f>
         <v>740</v>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="16" t="n">
         <f aca="false">$A13*$B$18*(E$4-$B$16)-$B$17</f>
         <v>830</v>
       </c>
-      <c r="F13" s="17" t="n">
+      <c r="F13" s="16" t="n">
         <f aca="false">$A13*$B$18*(F$4-$B$16)-$B$17</f>
         <v>920</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="27" t="n">
         <v>100</v>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="16" t="n">
         <f aca="false">$A14*$B$18*(B$4-$B$16)-$B$17</f>
         <v>640</v>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="16" t="n">
         <f aca="false">$A14*$B$18*(C$4-$B$16)-$B$17</f>
         <v>740</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="16" t="n">
         <f aca="false">$A14*$B$18*(D$4-$B$16)-$B$17</f>
         <v>840</v>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="16" t="n">
         <f aca="false">$A14*$B$18*(E$4-$B$16)-$B$17</f>
         <v>940</v>
       </c>
-      <c r="F14" s="17" t="n">
+      <c r="F14" s="16" t="n">
         <f aca="false">$A14*$B$18*(F$4-$B$16)-$B$17</f>
         <v>1040</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="14" t="n">
         <f aca="false">IF(Projection!C19=0,0,Projection!C15/Projection!C19)</f>
         <v>0</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="22" t="n">
+      <c r="B17" s="21" t="n">
         <f aca="false">Inputs!B17</f>
         <v>160</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="16" t="n">
+      <c r="B18" s="15" t="n">
         <f aca="false">Inputs!B20</f>
         <v>2</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>66</v>
       </c>
     </row>
@@ -2043,255 +2040,255 @@
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="32"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="str">
         <f aca="false">IF(Inputs!A5="","",Inputs!A5)</f>
         <v>Medhu Vadai</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="15" t="n">
         <f aca="false">Inputs!E5</f>
         <v>50</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="15" t="n">
         <f aca="false">Projection!E5</f>
         <v>40</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="15" t="n">
         <f aca="false">Projection!G5</f>
         <v>70</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E5" s="23" t="n">
         <f aca="false">IF(OR(A5="",Inputs!E5=""),0,B5-C5)</f>
         <v>10</v>
       </c>
-      <c r="F5" s="17" t="n">
+      <c r="F5" s="16" t="n">
         <f aca="false">B5*Inputs!C5</f>
         <v>300</v>
       </c>
-      <c r="G5" s="11" t="str">
+      <c r="G5" s="10" t="str">
         <f aca="false">IF(A5="","",IF(Inputs!E5="","Enter stock on Inputs",IF(B5&gt;=D5,"Enough even for a busy weekend",IF(B5&gt;=C5,"Enough for expected","Short by "&amp;(C5-B5)&amp;" for expected"))))</f>
         <v>Enough for expected</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="str">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="str">
         <f aca="false">IF(Inputs!A6="","",Inputs!A6)</f>
         <v>Paneer Puff</v>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="15" t="n">
         <f aca="false">Inputs!E6</f>
         <v>40</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="15" t="n">
         <f aca="false">Projection!E6</f>
         <v>40</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="15" t="n">
         <f aca="false">Projection!G6</f>
         <v>70</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="23" t="n">
         <f aca="false">IF(OR(A6="",Inputs!E6=""),0,B6-C6)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="17" t="n">
+      <c r="F6" s="16" t="n">
         <f aca="false">B6*Inputs!C6</f>
         <v>160</v>
       </c>
-      <c r="G6" s="11" t="str">
+      <c r="G6" s="10" t="str">
         <f aca="false">IF(A6="","",IF(Inputs!E6="","Enter stock on Inputs",IF(B6&gt;=D6,"Enough even for a busy weekend",IF(B6&gt;=C6,"Enough for expected","Short by "&amp;(C6-B6)&amp;" for expected"))))</f>
         <v>Enough for expected</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="str">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="str">
         <f aca="false">IF(Inputs!A7="","",Inputs!A7)</f>
         <v>Podi Idly</v>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="15" t="n">
         <f aca="false">Inputs!E7</f>
         <v>30</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="15" t="n">
         <f aca="false">Projection!E7</f>
         <v>30</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="15" t="n">
         <f aca="false">Projection!G7</f>
         <v>50</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="23" t="n">
         <f aca="false">IF(OR(A7="",Inputs!E7=""),0,B7-C7)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="17" t="n">
+      <c r="F7" s="16" t="n">
         <f aca="false">B7*Inputs!C7</f>
         <v>240</v>
       </c>
-      <c r="G7" s="11" t="str">
+      <c r="G7" s="10" t="str">
         <f aca="false">IF(A7="","",IF(Inputs!E7="","Enter stock on Inputs",IF(B7&gt;=D7,"Enough even for a busy weekend",IF(B7&gt;=C7,"Enough for expected","Short by "&amp;(C7-B7)&amp;" for expected"))))</f>
         <v>Enough for expected</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="str">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="str">
         <f aca="false">IF(Inputs!A8="","",Inputs!A8)</f>
         <v>Rose Milk</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="15" t="n">
         <f aca="false">Inputs!E8</f>
         <v>20</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="15" t="n">
         <f aca="false">Projection!E8</f>
         <v>50</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="15" t="n">
         <f aca="false">Projection!G8</f>
         <v>80</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="23" t="n">
         <f aca="false">IF(OR(A8="",Inputs!E8=""),0,B8-C8)</f>
         <v>-30</v>
       </c>
-      <c r="F8" s="17" t="n">
+      <c r="F8" s="16" t="n">
         <f aca="false">B8*Inputs!C8</f>
         <v>80</v>
       </c>
-      <c r="G8" s="11" t="str">
+      <c r="G8" s="10" t="str">
         <f aca="false">IF(A8="","",IF(Inputs!E8="","Enter stock on Inputs",IF(B8&gt;=D8,"Enough even for a busy weekend",IF(B8&gt;=C8,"Enough for expected","Short by "&amp;(C8-B8)&amp;" for expected"))))</f>
         <v>Short by 30 for expected</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="str">
         <f aca="false">IF(Inputs!A9="","",Inputs!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="15" t="n">
         <f aca="false">Inputs!E9</f>
         <v>0</v>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="15" t="n">
         <f aca="false">Projection!E9</f>
         <v>0</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="15" t="n">
         <f aca="false">Projection!G9</f>
         <v>0</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="23" t="n">
         <f aca="false">IF(OR(A9="",Inputs!E9=""),0,B9-C9)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="17" t="n">
+      <c r="F9" s="16" t="n">
         <f aca="false">B9*Inputs!C9</f>
         <v>0</v>
       </c>
-      <c r="G9" s="11" t="str">
+      <c r="G9" s="10" t="str">
         <f aca="false">IF(A9="","",IF(Inputs!E9="","Enter stock on Inputs",IF(B9&gt;=D9,"Enough even for a busy weekend",IF(B9&gt;=C9,"Enough for expected","Short by "&amp;(C9-B9)&amp;" for expected"))))</f>
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="str">
         <f aca="false">IF(Inputs!A10="","",Inputs!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="15" t="n">
         <f aca="false">Inputs!E10</f>
         <v>0</v>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="15" t="n">
         <f aca="false">Projection!E10</f>
         <v>0</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="15" t="n">
         <f aca="false">Projection!G10</f>
         <v>0</v>
       </c>
-      <c r="E10" s="24" t="n">
+      <c r="E10" s="23" t="n">
         <f aca="false">IF(OR(A10="",Inputs!E10=""),0,B10-C10)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="17" t="n">
+      <c r="F10" s="16" t="n">
         <f aca="false">B10*Inputs!C10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="11" t="str">
+      <c r="G10" s="10" t="str">
         <f aca="false">IF(A10="","",IF(Inputs!E10="","Enter stock on Inputs",IF(B10&gt;=D10,"Enough even for a busy weekend",IF(B10&gt;=C10,"Enough for expected","Short by "&amp;(C10-B10)&amp;" for expected"))))</f>
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="20" t="n">
+      <c r="B11" s="19" t="n">
         <f aca="false">SUM(B5:B10)</f>
         <v>140</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="19" t="n">
         <f aca="false">SUM(C5:C10)</f>
         <v>160</v>
       </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="19" t="n">
         <f aca="false">SUM(D5:D10)</f>
         <v>270</v>
       </c>
-      <c r="E11" s="20" t="n">
+      <c r="E11" s="19" t="n">
         <f aca="false">SUM(E5:E10)</f>
         <v>-20</v>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" s="20" t="n">
         <f aca="false">SUM(F5:F10)</f>
         <v>780</v>
       </c>
-      <c r="G11" s="19"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="G11" s="18"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2316,298 +2313,330 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="4" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="str">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="str">
         <f aca="false">IF(Inputs!A5="","",Inputs!A5)</f>
         <v>Medhu Vadai</v>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="14" t="n">
+        <f aca="false">Inputs!C5</f>
+        <v>6</v>
+      </c>
+      <c r="C5" s="15" t="n">
         <f aca="false">Projection!E5</f>
         <v>40</v>
       </c>
-      <c r="C5" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="D5" s="24" t="n">
-        <f aca="false">IF(C5="",0,C5-B5)</f>
-        <v>-22</v>
-      </c>
-      <c r="E5" s="22" t="n">
-        <f aca="false">Projection!F5</f>
+      <c r="D5" s="9"/>
+      <c r="E5" s="23" t="n">
+        <f aca="false">IF(D5="",0,D5-C5)</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <f aca="false">B5*C5</f>
         <v>240</v>
       </c>
-      <c r="F5" s="17" t="n">
-        <f aca="false">N(C5)*Inputs!C5</f>
-        <v>108</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="str">
+      <c r="G5" s="16" t="n">
+        <f aca="false">B5*D5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="str">
         <f aca="false">IF(Inputs!A6="","",Inputs!A6)</f>
         <v>Paneer Puff</v>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="14" t="n">
+        <f aca="false">Inputs!C6</f>
+        <v>4</v>
+      </c>
+      <c r="C6" s="15" t="n">
         <f aca="false">Projection!E6</f>
         <v>40</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="24" t="n">
-        <f aca="false">IF(C6="",0,C6-B6)</f>
-        <v>0</v>
-      </c>
-      <c r="E6" s="22" t="n">
-        <f aca="false">Projection!F6</f>
+      <c r="D6" s="9"/>
+      <c r="E6" s="23" t="n">
+        <f aca="false">IF(D6="",0,D6-C6)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <f aca="false">B6*C6</f>
         <v>160</v>
       </c>
-      <c r="F6" s="17" t="n">
-        <f aca="false">N(C6)*Inputs!C6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="str">
+      <c r="G6" s="16" t="n">
+        <f aca="false">B6*D6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="str">
         <f aca="false">IF(Inputs!A7="","",Inputs!A7)</f>
         <v>Podi Idly</v>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="14" t="n">
+        <f aca="false">Inputs!C7</f>
+        <v>8</v>
+      </c>
+      <c r="C7" s="15" t="n">
         <f aca="false">Projection!E7</f>
         <v>30</v>
       </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="24" t="n">
-        <f aca="false">IF(C7="",0,C7-B7)</f>
-        <v>0</v>
-      </c>
-      <c r="E7" s="22" t="n">
-        <f aca="false">Projection!F7</f>
+      <c r="D7" s="9"/>
+      <c r="E7" s="23" t="n">
+        <f aca="false">IF(D7="",0,D7-C7)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <f aca="false">B7*C7</f>
         <v>240</v>
       </c>
-      <c r="F7" s="17" t="n">
-        <f aca="false">N(C7)*Inputs!C7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="str">
+      <c r="G7" s="16" t="n">
+        <f aca="false">B7*D7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="str">
         <f aca="false">IF(Inputs!A8="","",Inputs!A8)</f>
         <v>Rose Milk</v>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="14" t="n">
+        <f aca="false">Inputs!C8</f>
+        <v>4</v>
+      </c>
+      <c r="C8" s="15" t="n">
         <f aca="false">Projection!E8</f>
         <v>50</v>
       </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="24" t="n">
-        <f aca="false">IF(C8="",0,C8-B8)</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="22" t="n">
-        <f aca="false">Projection!F8</f>
+      <c r="D8" s="9"/>
+      <c r="E8" s="23" t="n">
+        <f aca="false">IF(D8="",0,D8-C8)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <f aca="false">B8*C8</f>
         <v>200</v>
       </c>
-      <c r="F8" s="17" t="n">
-        <f aca="false">N(C8)*Inputs!C8</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="str">
+      <c r="G8" s="16" t="n">
+        <f aca="false">B8*D8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="str">
         <f aca="false">IF(Inputs!A9="","",Inputs!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="14" t="n">
+        <f aca="false">Inputs!C9</f>
+        <v>0</v>
+      </c>
+      <c r="C9" s="15" t="n">
         <f aca="false">Projection!E9</f>
         <v>0</v>
       </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="24" t="n">
-        <f aca="false">IF(C9="",0,C9-B9)</f>
-        <v>0</v>
-      </c>
-      <c r="E9" s="22" t="n">
-        <f aca="false">Projection!F9</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="17" t="n">
-        <f aca="false">N(C9)*Inputs!C9</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="str">
+      <c r="D9" s="8"/>
+      <c r="E9" s="23" t="n">
+        <f aca="false">IF(D9="",0,D9-C9)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <f aca="false">B9*C9</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <f aca="false">B9*D9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="str">
         <f aca="false">IF(Inputs!A10="","",Inputs!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="14" t="n">
+        <f aca="false">Inputs!C10</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="15" t="n">
         <f aca="false">Projection!E10</f>
         <v>0</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="24" t="n">
-        <f aca="false">IF(C10="",0,C10-B10)</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="22" t="n">
-        <f aca="false">Projection!F10</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="17" t="n">
-        <f aca="false">N(C10)*Inputs!C10</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
+      <c r="D10" s="8"/>
+      <c r="E10" s="23" t="n">
+        <f aca="false">IF(D10="",0,D10-C10)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <f aca="false">B10*C10</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <f aca="false">B10*D10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="20" t="n">
-        <f aca="false">SUM(B5:B10)</f>
+      <c r="B11" s="18"/>
+      <c r="C11" s="19" t="n">
+        <f aca="false">SUM(C5:C10)</f>
         <v>160</v>
       </c>
-      <c r="C11" s="20" t="n">
-        <f aca="false">SUM(C5:C10)</f>
-        <v>18</v>
-      </c>
-      <c r="D11" s="20" t="n">
+      <c r="D11" s="19" t="n">
         <f aca="false">SUM(D5:D10)</f>
-        <v>-22</v>
-      </c>
-      <c r="E11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="19" t="n">
         <f aca="false">SUM(E5:E10)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <f aca="false">SUM(F5:F10)</f>
         <v>840</v>
       </c>
-      <c r="F11" s="21" t="n">
-        <f aca="false">SUM(F5:F10)</f>
-        <v>108</v>
+      <c r="G11" s="20" t="n">
+        <f aca="false">SUM(G5:G10)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="5" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <f aca="false">F11</f>
+        <v>840</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <f aca="false">G11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="21" t="n">
+        <f aca="false">Projection!C15</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <f aca="false">SUMPRODUCT(D5:D10,Inputs!$D$5:$D$10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="17" t="n">
-        <f aca="false">E11</f>
-        <v>840</v>
-      </c>
-      <c r="C14" s="17" t="n">
-        <f aca="false">F11</f>
-        <v>108</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="22" t="n">
-        <f aca="false">Projection!C15</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="17" t="n">
-        <f aca="false">SUMPRODUCT(C5:C10,Inputs!$D$5:$D$10)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="21" t="n">
         <f aca="false">Inputs!B17</f>
         <v>160</v>
       </c>
-      <c r="C16" s="29" t="n">
+      <c r="C16" s="28" t="n">
         <f aca="false">Inputs!B17</f>
         <v>160</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+      <c r="D16" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="20" t="n">
         <f aca="false">B14-B15-B16</f>
         <v>680</v>
       </c>
-      <c r="C17" s="21" t="n">
+      <c r="C17" s="20" t="n">
         <f aca="false">C14-C15-C16</f>
-        <v>-52</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+        <v>-160</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <f aca="false">C17-B17</f>
+        <v>-840</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C18" s="17" t="n">
-        <f aca="false">C17-B17</f>
-        <v>-732</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D5:D11">
+  <conditionalFormatting sqref="E5:E11">
     <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C18">
-    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+  <conditionalFormatting sqref="B17:C18">
+    <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B17:C17">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Fill projection Actuals with real sales from the ledger
Units sold (16/21/8/8/1), real spend $144, updated Rose Milk price,
stock counts and the Misc item to match the tracker.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RGZwPX49EKhhzekY9w6486
</commit_message>
<xml_diff>
--- a/stall/Stall_Sales_Projection.xlsx
+++ b/stall/Stall_Sales_Projection.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="86">
   <si>
     <t xml:space="preserve">Snack Stall: Projection Inputs</t>
   </si>
@@ -87,7 +87,7 @@
     <t xml:space="preserve">1 plate</t>
   </si>
   <si>
-    <t xml:space="preserve">Prices: from you (Idly $8 and Rose Milk $4, as updated in the tracker).</t>
+    <t xml:space="preserve">Prices: from the tracker (Rose Milk $3, Misc $3 as sold).</t>
   </si>
   <si>
     <t xml:space="preserve">Paneer Puff</t>
@@ -102,7 +102,7 @@
     <t xml:space="preserve">Podi Idly</t>
   </si>
   <si>
-    <t xml:space="preserve">Stock: from you (50 / 40 / 30 / 20 for the weekend).</t>
+    <t xml:space="preserve">Stock: from the tracker (50 / 30 / 20 / 15; Misc not counted).</t>
   </si>
   <si>
     <t xml:space="preserve">Rose Milk</t>
@@ -114,7 +114,10 @@
     <t xml:space="preserve">Ingredient cost: 0 because your $50 cooking items are in fixed costs. Enter a per-unit cost to model buying more for bigger days.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rows 9-10: spare rows for new items.</t>
+    <t xml:space="preserve">Misc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misc: added in the tracker during the event. Row 10 is a spare row.</t>
   </si>
   <si>
     <t xml:space="preserve">Fixed costs</t>
@@ -273,7 +276,7 @@
     <t xml:space="preserve">Actuals vs Projection</t>
   </si>
   <si>
-    <t xml:space="preserve">After the weekend, enter units sold from the tracker's Summary export (the Sold column). Actual sales = price x units sold. Yellow cells are yours to fill.</t>
+    <t xml:space="preserve">Units sold are from the tracker (31 orders, exported Oct 12). Actual sales = price x units sold. Yellow cells can be changed if more sales come in.</t>
   </si>
   <si>
     <t xml:space="preserve">Actual units sold</t>
@@ -295,13 +298,13 @@
     <t xml:space="preserve">Spend</t>
   </si>
   <si>
-    <t xml:space="preserve">Type over this with your real total spend from the tracker if it changed.</t>
+    <t xml:space="preserve">Real spend from the tracker: stall fee $60, supplies $38, cooking items $45, Drift $1.</t>
   </si>
   <si>
     <t xml:space="preserve">Actual vs expected</t>
   </si>
   <si>
-    <t xml:space="preserve">Leave Actual units blank until the weekend is done. Until then, Actual shows a loss of your spend.</t>
+    <t xml:space="preserve">Expected uses the Inputs guesses; Actual uses what the tracker recorded.</t>
   </si>
 </sst>
 </file>
@@ -585,7 +588,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -979,7 +982,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F6" s="9" t="n">
         <v>10</v>
@@ -1008,7 +1011,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>8</v>
@@ -1031,13 +1034,13 @@
         <v>20</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F8" s="9" t="n">
         <v>12</v>
@@ -1053,16 +1056,28 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5"/>
+      <c r="A9" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="B9" s="5"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
+      <c r="C9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
+      <c r="F9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="I9" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1077,59 +1092,59 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="6" t="n">
         <v>60</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>50</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B15" s="6" t="n">
         <v>50</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B16" s="6" t="n">
         <v>0</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">SUM(B13:B16)</f>
@@ -1138,29 +1153,29 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B21" s="9" t="n">
         <v>6</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1193,12 +1208,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1209,22 +1224,22 @@
         <v>4</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1336,7 +1351,7 @@
       </c>
       <c r="B8" s="14" t="n">
         <f aca="false">Inputs!C8</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8" s="15" t="n">
         <f aca="false">Inputs!F8*Inputs!$B$20</f>
@@ -1344,7 +1359,7 @@
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">C8*$B8</f>
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">Inputs!G8*Inputs!$B$20</f>
@@ -1352,7 +1367,7 @@
       </c>
       <c r="F8" s="16" t="n">
         <f aca="false">E8*$B8</f>
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G8" s="15" t="n">
         <f aca="false">Inputs!H8*Inputs!$B$20</f>
@@ -1360,17 +1375,17 @@
       </c>
       <c r="H8" s="16" t="n">
         <f aca="false">G8*$B8</f>
-        <v>320</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="str">
         <f aca="false">IF(Inputs!A9="","",Inputs!A9)</f>
-        <v/>
+        <v>Misc</v>
       </c>
       <c r="B9" s="14" t="n">
         <f aca="false">Inputs!C9</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C9" s="15" t="n">
         <f aca="false">Inputs!F9*Inputs!$B$20</f>
@@ -1433,7 +1448,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="19" t="n">
@@ -1442,7 +1457,7 @@
       </c>
       <c r="D11" s="20" t="n">
         <f aca="false">SUM(D5:D10)</f>
-        <v>424</v>
+        <v>400</v>
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">SUM(E5:E10)</f>
@@ -1450,7 +1465,7 @@
       </c>
       <c r="F11" s="20" t="n">
         <f aca="false">SUM(F5:F10)</f>
-        <v>840</v>
+        <v>790</v>
       </c>
       <c r="G11" s="19" t="n">
         <f aca="false">SUM(G5:G10)</f>
@@ -1458,43 +1473,43 @@
       </c>
       <c r="H11" s="20" t="n">
         <f aca="false">SUM(H5:H10)</f>
-        <v>1420</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B14" s="16" t="n">
         <f aca="false">D11</f>
-        <v>424</v>
+        <v>400</v>
       </c>
       <c r="C14" s="16" t="n">
         <f aca="false">F11</f>
-        <v>840</v>
+        <v>790</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">H11</f>
-        <v>1420</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B15" s="16" t="n">
         <f aca="false">SUMPRODUCT(C5:C10,Inputs!$D$5:$D$10)</f>
@@ -1511,7 +1526,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16" s="21" t="n">
         <f aca="false">Inputs!$B$17</f>
@@ -1528,41 +1543,41 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B17" s="20" t="n">
         <f aca="false">B14-B15-B16</f>
-        <v>264</v>
+        <v>240</v>
       </c>
       <c r="C17" s="20" t="n">
         <f aca="false">C14-C15-C16</f>
-        <v>680</v>
+        <v>630</v>
       </c>
       <c r="D17" s="20" t="n">
         <f aca="false">D14-D15-D16</f>
-        <v>1260</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B18" s="22" t="n">
         <f aca="false">IF(B14=0,0,B17/B14)</f>
-        <v>0.622641509433962</v>
+        <v>0.6</v>
       </c>
       <c r="C18" s="22" t="n">
         <f aca="false">IF(C14=0,0,C17/C14)</f>
-        <v>0.80952380952381</v>
+        <v>0.79746835443038</v>
       </c>
       <c r="D18" s="22" t="n">
         <f aca="false">IF(D14=0,0,D17/D14)</f>
-        <v>0.887323943661972</v>
+        <v>0.880597014925373</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B19" s="23" t="n">
         <f aca="false">C11</f>
@@ -1579,7 +1594,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B20" s="24" t="n">
         <f aca="false">IF(Inputs!$B$20*Inputs!$B$21=0,0,B19/(Inputs!$B$20*Inputs!$B$21))</f>
@@ -1596,75 +1611,75 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B21" s="25" t="n">
         <f aca="false">IF(B19=0,0,B14/B19)</f>
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="C21" s="25" t="n">
         <f aca="false">IF(C19=0,0,C14/C19)</f>
-        <v>5.25</v>
+        <v>4.9375</v>
       </c>
       <c r="D21" s="25" t="n">
         <f aca="false">IF(D19=0,0,D14/D19)</f>
-        <v>5.25925925925926</v>
+        <v>4.96296296296296</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B22" s="25" t="n">
         <f aca="false">IF(B19=0,0,(B14-B15)/B19)</f>
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="C22" s="25" t="n">
         <f aca="false">IF(C19=0,0,(C14-C15)/C19)</f>
-        <v>5.25</v>
+        <v>4.9375</v>
       </c>
       <c r="D22" s="25" t="n">
         <f aca="false">IF(D19=0,0,(D14-D15)/D19)</f>
-        <v>5.25925925925926</v>
+        <v>4.96296296296296</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B23" s="23" t="n">
         <f aca="false">IF(B22&lt;=0,0,ROUNDUP(Inputs!$B$17/B22,0))</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C23" s="23" t="n">
         <f aca="false">IF(C22&lt;=0,0,ROUNDUP(Inputs!$B$17/C22,0))</f>
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D23" s="23" t="n">
         <f aca="false">IF(D22&lt;=0,0,ROUNDUP(Inputs!$B$17/D22,0))</f>
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B24" s="16" t="n">
         <f aca="false">B23*B21</f>
-        <v>164.3</v>
+        <v>160</v>
       </c>
       <c r="C24" s="16" t="n">
         <f aca="false">C23*C21</f>
-        <v>162.75</v>
+        <v>162.9375</v>
       </c>
       <c r="D24" s="16" t="n">
         <f aca="false">D23*D21</f>
-        <v>163.037037037037</v>
+        <v>163.777777777778</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1700,17 +1715,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" s="26" t="n">
         <v>4</v>
@@ -1980,19 +1995,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B16" s="14" t="n">
         <f aca="false">IF(Projection!C19=0,0,Projection!C15/Projection!C19)</f>
         <v>0</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B17" s="21" t="n">
         <f aca="false">Inputs!B17</f>
@@ -2001,7 +2016,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18" s="15" t="n">
         <f aca="false">Inputs!B20</f>
@@ -2010,7 +2025,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -2050,12 +2065,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2063,22 +2078,22 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2107,7 +2122,7 @@
         <v>300</v>
       </c>
       <c r="G5" s="10" t="str">
-        <f aca="false">IF(A5="","",IF(Inputs!E5="","Enter stock on Inputs",IF(B5&gt;=D5,"Enough even for a busy weekend",IF(B5&gt;=C5,"Enough for expected","Short by "&amp;(C5-B5)&amp;" for expected"))))</f>
+        <f aca="false">IF(A5="","",IF(Inputs!E5="","Stock not counted",IF(B5&gt;=D5,"Enough even for a busy weekend",IF(B5&gt;=C5,"Enough for expected","Short by "&amp;(C5-B5)&amp;" for expected"))))</f>
         <v>Enough for expected</v>
       </c>
     </row>
@@ -2118,7 +2133,7 @@
       </c>
       <c r="B6" s="15" t="n">
         <f aca="false">Inputs!E6</f>
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C6" s="15" t="n">
         <f aca="false">Projection!E6</f>
@@ -2130,15 +2145,15 @@
       </c>
       <c r="E6" s="23" t="n">
         <f aca="false">IF(OR(A6="",Inputs!E6=""),0,B6-C6)</f>
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="F6" s="16" t="n">
         <f aca="false">B6*Inputs!C6</f>
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="G6" s="10" t="str">
-        <f aca="false">IF(A6="","",IF(Inputs!E6="","Enter stock on Inputs",IF(B6&gt;=D6,"Enough even for a busy weekend",IF(B6&gt;=C6,"Enough for expected","Short by "&amp;(C6-B6)&amp;" for expected"))))</f>
-        <v>Enough for expected</v>
+        <f aca="false">IF(A6="","",IF(Inputs!E6="","Stock not counted",IF(B6&gt;=D6,"Enough even for a busy weekend",IF(B6&gt;=C6,"Enough for expected","Short by "&amp;(C6-B6)&amp;" for expected"))))</f>
+        <v>Short by 10 for expected</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2148,7 +2163,7 @@
       </c>
       <c r="B7" s="15" t="n">
         <f aca="false">Inputs!E7</f>
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C7" s="15" t="n">
         <f aca="false">Projection!E7</f>
@@ -2160,15 +2175,15 @@
       </c>
       <c r="E7" s="23" t="n">
         <f aca="false">IF(OR(A7="",Inputs!E7=""),0,B7-C7)</f>
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="F7" s="16" t="n">
         <f aca="false">B7*Inputs!C7</f>
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="G7" s="10" t="str">
-        <f aca="false">IF(A7="","",IF(Inputs!E7="","Enter stock on Inputs",IF(B7&gt;=D7,"Enough even for a busy weekend",IF(B7&gt;=C7,"Enough for expected","Short by "&amp;(C7-B7)&amp;" for expected"))))</f>
-        <v>Enough for expected</v>
+        <f aca="false">IF(A7="","",IF(Inputs!E7="","Stock not counted",IF(B7&gt;=D7,"Enough even for a busy weekend",IF(B7&gt;=C7,"Enough for expected","Short by "&amp;(C7-B7)&amp;" for expected"))))</f>
+        <v>Short by 10 for expected</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2178,7 +2193,7 @@
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">Inputs!E8</f>
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C8" s="15" t="n">
         <f aca="false">Projection!E8</f>
@@ -2190,21 +2205,21 @@
       </c>
       <c r="E8" s="23" t="n">
         <f aca="false">IF(OR(A8="",Inputs!E8=""),0,B8-C8)</f>
-        <v>-30</v>
+        <v>-35</v>
       </c>
       <c r="F8" s="16" t="n">
         <f aca="false">B8*Inputs!C8</f>
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="G8" s="10" t="str">
-        <f aca="false">IF(A8="","",IF(Inputs!E8="","Enter stock on Inputs",IF(B8&gt;=D8,"Enough even for a busy weekend",IF(B8&gt;=C8,"Enough for expected","Short by "&amp;(C8-B8)&amp;" for expected"))))</f>
-        <v>Short by 30 for expected</v>
+        <f aca="false">IF(A8="","",IF(Inputs!E8="","Stock not counted",IF(B8&gt;=D8,"Enough even for a busy weekend",IF(B8&gt;=C8,"Enough for expected","Short by "&amp;(C8-B8)&amp;" for expected"))))</f>
+        <v>Short by 35 for expected</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="str">
         <f aca="false">IF(Inputs!A9="","",Inputs!A9)</f>
-        <v/>
+        <v>Misc</v>
       </c>
       <c r="B9" s="15" t="n">
         <f aca="false">Inputs!E9</f>
@@ -2227,8 +2242,8 @@
         <v>0</v>
       </c>
       <c r="G9" s="10" t="str">
-        <f aca="false">IF(A9="","",IF(Inputs!E9="","Enter stock on Inputs",IF(B9&gt;=D9,"Enough even for a busy weekend",IF(B9&gt;=C9,"Enough for expected","Short by "&amp;(C9-B9)&amp;" for expected"))))</f>
-        <v/>
+        <f aca="false">IF(A9="","",IF(Inputs!E9="","Stock not counted",IF(B9&gt;=D9,"Enough even for a busy weekend",IF(B9&gt;=C9,"Enough for expected","Short by "&amp;(C9-B9)&amp;" for expected"))))</f>
+        <v>Stock not counted</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2257,17 +2272,17 @@
         <v>0</v>
       </c>
       <c r="G10" s="10" t="str">
-        <f aca="false">IF(A10="","",IF(Inputs!E10="","Enter stock on Inputs",IF(B10&gt;=D10,"Enough even for a busy weekend",IF(B10&gt;=C10,"Enough for expected","Short by "&amp;(C10-B10)&amp;" for expected"))))</f>
+        <f aca="false">IF(A10="","",IF(Inputs!E10="","Stock not counted",IF(B10&gt;=D10,"Enough even for a busy weekend",IF(B10&gt;=C10,"Enough for expected","Short by "&amp;(C10-B10)&amp;" for expected"))))</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="false">SUM(B5:B10)</f>
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="C11" s="19" t="n">
         <f aca="false">SUM(C5:C10)</f>
@@ -2279,17 +2294,17 @@
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">SUM(E5:E10)</f>
-        <v>-20</v>
+        <v>-45</v>
       </c>
       <c r="F11" s="20" t="n">
         <f aca="false">SUM(F5:F10)</f>
-        <v>780</v>
+        <v>625</v>
       </c>
       <c r="G11" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -2325,12 +2340,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2341,19 +2356,19 @@
         <v>4</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2369,10 +2384,12 @@
         <f aca="false">Projection!E5</f>
         <v>40</v>
       </c>
-      <c r="D5" s="9"/>
+      <c r="D5" s="9" t="n">
+        <v>16</v>
+      </c>
       <c r="E5" s="23" t="n">
         <f aca="false">IF(D5="",0,D5-C5)</f>
-        <v>0</v>
+        <v>-24</v>
       </c>
       <c r="F5" s="16" t="n">
         <f aca="false">B5*C5</f>
@@ -2380,7 +2397,7 @@
       </c>
       <c r="G5" s="16" t="n">
         <f aca="false">B5*D5</f>
-        <v>0</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2396,10 +2413,12 @@
         <f aca="false">Projection!E6</f>
         <v>40</v>
       </c>
-      <c r="D6" s="9"/>
+      <c r="D6" s="9" t="n">
+        <v>21</v>
+      </c>
       <c r="E6" s="23" t="n">
         <f aca="false">IF(D6="",0,D6-C6)</f>
-        <v>0</v>
+        <v>-19</v>
       </c>
       <c r="F6" s="16" t="n">
         <f aca="false">B6*C6</f>
@@ -2407,7 +2426,7 @@
       </c>
       <c r="G6" s="16" t="n">
         <f aca="false">B6*D6</f>
-        <v>0</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2423,10 +2442,12 @@
         <f aca="false">Projection!E7</f>
         <v>30</v>
       </c>
-      <c r="D7" s="9"/>
+      <c r="D7" s="9" t="n">
+        <v>8</v>
+      </c>
       <c r="E7" s="23" t="n">
         <f aca="false">IF(D7="",0,D7-C7)</f>
-        <v>0</v>
+        <v>-22</v>
       </c>
       <c r="F7" s="16" t="n">
         <f aca="false">B7*C7</f>
@@ -2434,7 +2455,7 @@
       </c>
       <c r="G7" s="16" t="n">
         <f aca="false">B7*D7</f>
-        <v>0</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2444,43 +2465,47 @@
       </c>
       <c r="B8" s="14" t="n">
         <f aca="false">Inputs!C8</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8" s="15" t="n">
         <f aca="false">Projection!E8</f>
         <v>50</v>
       </c>
-      <c r="D8" s="9"/>
+      <c r="D8" s="9" t="n">
+        <v>8</v>
+      </c>
       <c r="E8" s="23" t="n">
         <f aca="false">IF(D8="",0,D8-C8)</f>
-        <v>0</v>
+        <v>-42</v>
       </c>
       <c r="F8" s="16" t="n">
         <f aca="false">B8*C8</f>
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">B8*D8</f>
-        <v>0</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="str">
         <f aca="false">IF(Inputs!A9="","",Inputs!A9)</f>
-        <v/>
+        <v>Misc</v>
       </c>
       <c r="B9" s="14" t="n">
         <f aca="false">Inputs!C9</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C9" s="15" t="n">
         <f aca="false">Projection!E9</f>
         <v>0</v>
       </c>
-      <c r="D9" s="8"/>
+      <c r="D9" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="E9" s="23" t="n">
         <f aca="false">IF(D9="",0,D9-C9)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="16" t="n">
         <f aca="false">B9*C9</f>
@@ -2488,7 +2513,7 @@
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">B9*D9</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2520,7 +2545,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="18"/>
       <c r="C11" s="19" t="n">
@@ -2529,48 +2554,48 @@
       </c>
       <c r="D11" s="19" t="n">
         <f aca="false">SUM(D5:D10)</f>
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">SUM(E5:E10)</f>
-        <v>0</v>
+        <v>-106</v>
       </c>
       <c r="F11" s="20" t="n">
         <f aca="false">SUM(F5:F10)</f>
-        <v>840</v>
+        <v>790</v>
       </c>
       <c r="G11" s="20" t="n">
         <f aca="false">SUM(G5:G10)</f>
-        <v>0</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B14" s="16" t="n">
         <f aca="false">F11</f>
-        <v>840</v>
+        <v>790</v>
       </c>
       <c r="C14" s="16" t="n">
         <f aca="false">G11</f>
-        <v>0</v>
+        <v>271</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B15" s="21" t="n">
         <f aca="false">Projection!C15</f>
@@ -2583,45 +2608,44 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B16" s="21" t="n">
         <f aca="false">Inputs!B17</f>
         <v>160</v>
       </c>
       <c r="C16" s="28" t="n">
-        <f aca="false">Inputs!B17</f>
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B17" s="20" t="n">
         <f aca="false">B14-B15-B16</f>
-        <v>680</v>
+        <v>630</v>
       </c>
       <c r="C17" s="20" t="n">
         <f aca="false">C14-C15-C16</f>
-        <v>-160</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C18" s="16" t="n">
         <f aca="false">C17-B17</f>
-        <v>-840</v>
+        <v>-503</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Show profit margin in the tracker and the projection Actuals
Tracker: margin (profit / income) under Profit in the top bar, online
and offline. Workbook: Profit margin row on Actuals for expected and
actual.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RGZwPX49EKhhzekY9w6486
</commit_message>
<xml_diff>
--- a/stall/Stall_Sales_Projection.xlsx
+++ b/stall/Stall_Sales_Projection.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="87">
   <si>
     <t xml:space="preserve">Snack Stall: Projection Inputs</t>
   </si>
@@ -301,7 +301,10 @@
     <t xml:space="preserve">Real spend from the tracker: stall fee $60, supplies $38, cooking items $45, Drift $1.</t>
   </si>
   <si>
-    <t xml:space="preserve">Actual vs expected</t>
+    <t xml:space="preserve">Profit / sales: the share of each dollar of sales you kept.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actual vs expected profit</t>
   </si>
   <si>
     <t xml:space="preserve">Expected uses the Inputs guesses; Actual uses what the tracker recorded.</t>
@@ -2636,16 +2639,32 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="22" t="n">
+        <f aca="false">IF(B14=0,0,B17/B14)</f>
+        <v>0.79746835443038</v>
+      </c>
+      <c r="C18" s="22" t="n">
+        <f aca="false">IF(C14=0,0,C17/C14)</f>
+        <v>0.468634686346863</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C18" s="16" t="n">
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" s="16" t="n">
         <f aca="false">C17-B17</f>
         <v>-503</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -2654,13 +2673,18 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B17:C18">
+  <conditionalFormatting sqref="C19">
     <cfRule type="cellIs" priority="3" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B17:C18">
+    <cfRule type="cellIs" priority="4" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B17:C17">
-    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="5" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>